<commit_message>
summary statistics initiated, data cleaning file created and first filters added. variable vectors for selection and filtering saved, functions file created
</commit_message>
<xml_diff>
--- a/doc/CBCL_table_t_per_item.xlsx
+++ b/doc/CBCL_table_t_per_item.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CBCL_1</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J2">
@@ -484,7 +484,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CBCL_100</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J3">
@@ -524,7 +524,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CBCL_101</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J4">
@@ -564,7 +564,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CBCL_102</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J5">
@@ -614,7 +614,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CBCL_103</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J6">
@@ -659,7 +659,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CBCL_104</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J7">
@@ -699,7 +699,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CBCL_105</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J8">
@@ -734,7 +734,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CBCL_109</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J9">
@@ -774,7 +774,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CBCL_110</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J10">
@@ -819,7 +819,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CBCL_112</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J11">
@@ -859,7 +859,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CBCL_12</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J12">
@@ -899,7 +899,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CBCL_13</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J13">
@@ -939,7 +939,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CBCL_14</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J14">
@@ -979,7 +979,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CBCL_17</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J15">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>CBCL_18</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J16">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CBCL_19</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J17">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>CBCL_20</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J18">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>CBCL_21</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J19">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>CBCL_22</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J20">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CBCL_23</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J21">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>CBCL_24</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J22">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CBCL_25</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J23">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>CBCL_26</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J24">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CBCL_27</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J25">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>CBCL_28</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J26">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CBCL_29</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J27">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>CBCL_2</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J28">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CBCL_3</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J29">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>CBCL_30</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J30">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>CBCL_31</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J31">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>CBCL_32</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J32">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CBCL_33</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J33">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>CBCL_34</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J34">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CBCL_35</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J35">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>CBCL_37</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J36">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CBCL_38</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J37">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>CBCL_39</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J38">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>CBCL_41</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J39">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>CBCL_42</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J40">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>CBCL_43</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J41">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>CBCL_44</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J42">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CBCL_45</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J43">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>CBCL_46</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J44">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CBCL_47</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J45">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>CBCL_48</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J46">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>CBCL_49</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J47">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>CBCL_4</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J48">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>CBCL_50</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J49">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>CBCL_51</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J50">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>CBCL_52</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J51">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>CBCL_56c</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J52">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>CBCL_56d</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J53">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>CBCL_56e</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J54">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>CBCL_56f</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J55">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>CBCL_56g</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J56">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>CBCL_57</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J57">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>CBCL_58</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J58">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>CBCL_5</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J59">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>CBCL_61</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J60">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>CBCL_63</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J61">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>CBCL_64</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J62">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>CBCL_65</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J63">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>CBCL_66</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J64">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>CBCL_67</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J65">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>CBCL_68</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J66">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>CBCL_69</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J67">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>CBCL_7</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J68">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>CBCL_71</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J69">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>CBCL_72</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J70">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>CBCL_74</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J71">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>CBCL_75</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J72">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>CBCL_76</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J73">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>CBCL_77</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J74">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>CBCL_78</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J75">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>CBCL_80</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J76">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>CBCL_81</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J77">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>CBCL_82</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J78">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>CBCL_84</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J79">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>CBCL_89</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J80">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>CBCL_90</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J81">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>CBCL_91</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J82">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>CBCL_93</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J83">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>CBCL_94</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J84">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>CBCL_95</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J85">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>CBCL_96</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J86">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>CBCL_97</t>
+          <t>//1_//2</t>
         </is>
       </c>
       <c r="J87">

</xml_diff>

<commit_message>
plots created, summary statistics inspected
</commit_message>
<xml_diff>
--- a/doc/CBCL_table_t_per_item.xlsx
+++ b/doc/CBCL_table_t_per_item.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_1</t>
         </is>
       </c>
       <c r="J2">
@@ -484,7 +484,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_100</t>
         </is>
       </c>
       <c r="J3">
@@ -524,7 +524,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_101</t>
         </is>
       </c>
       <c r="J4">
@@ -564,7 +564,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_102</t>
         </is>
       </c>
       <c r="J5">
@@ -614,7 +614,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_103</t>
         </is>
       </c>
       <c r="J6">
@@ -659,7 +659,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_104</t>
         </is>
       </c>
       <c r="J7">
@@ -699,7 +699,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_105</t>
         </is>
       </c>
       <c r="J8">
@@ -734,7 +734,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_109</t>
         </is>
       </c>
       <c r="J9">
@@ -774,7 +774,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_110</t>
         </is>
       </c>
       <c r="J10">
@@ -819,7 +819,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_112</t>
         </is>
       </c>
       <c r="J11">
@@ -859,7 +859,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_12</t>
         </is>
       </c>
       <c r="J12">
@@ -899,7 +899,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_13</t>
         </is>
       </c>
       <c r="J13">
@@ -939,7 +939,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_14</t>
         </is>
       </c>
       <c r="J14">
@@ -979,7 +979,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_17</t>
         </is>
       </c>
       <c r="J15">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_18</t>
         </is>
       </c>
       <c r="J16">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_19</t>
         </is>
       </c>
       <c r="J17">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_20</t>
         </is>
       </c>
       <c r="J18">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_21</t>
         </is>
       </c>
       <c r="J19">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_22</t>
         </is>
       </c>
       <c r="J20">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_23</t>
         </is>
       </c>
       <c r="J21">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_24</t>
         </is>
       </c>
       <c r="J22">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_25</t>
         </is>
       </c>
       <c r="J23">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_26</t>
         </is>
       </c>
       <c r="J24">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_27</t>
         </is>
       </c>
       <c r="J25">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_28</t>
         </is>
       </c>
       <c r="J26">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_29</t>
         </is>
       </c>
       <c r="J27">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_2</t>
         </is>
       </c>
       <c r="J28">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_3</t>
         </is>
       </c>
       <c r="J29">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_30</t>
         </is>
       </c>
       <c r="J30">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_31</t>
         </is>
       </c>
       <c r="J31">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_32</t>
         </is>
       </c>
       <c r="J32">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_33</t>
         </is>
       </c>
       <c r="J33">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_34</t>
         </is>
       </c>
       <c r="J34">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_35</t>
         </is>
       </c>
       <c r="J35">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_37</t>
         </is>
       </c>
       <c r="J36">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_38</t>
         </is>
       </c>
       <c r="J37">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_39</t>
         </is>
       </c>
       <c r="J38">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_41</t>
         </is>
       </c>
       <c r="J39">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_42</t>
         </is>
       </c>
       <c r="J40">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_43</t>
         </is>
       </c>
       <c r="J41">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_44</t>
         </is>
       </c>
       <c r="J42">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_45</t>
         </is>
       </c>
       <c r="J43">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_46</t>
         </is>
       </c>
       <c r="J44">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_47</t>
         </is>
       </c>
       <c r="J45">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_48</t>
         </is>
       </c>
       <c r="J46">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_49</t>
         </is>
       </c>
       <c r="J47">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_4</t>
         </is>
       </c>
       <c r="J48">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_50</t>
         </is>
       </c>
       <c r="J49">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_51</t>
         </is>
       </c>
       <c r="J50">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_52</t>
         </is>
       </c>
       <c r="J51">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_56c</t>
         </is>
       </c>
       <c r="J52">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_56d</t>
         </is>
       </c>
       <c r="J53">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_56e</t>
         </is>
       </c>
       <c r="J54">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_56f</t>
         </is>
       </c>
       <c r="J55">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_56g</t>
         </is>
       </c>
       <c r="J56">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_57</t>
         </is>
       </c>
       <c r="J57">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_58</t>
         </is>
       </c>
       <c r="J58">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_5</t>
         </is>
       </c>
       <c r="J59">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_61</t>
         </is>
       </c>
       <c r="J60">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_63</t>
         </is>
       </c>
       <c r="J61">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_64</t>
         </is>
       </c>
       <c r="J62">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_65</t>
         </is>
       </c>
       <c r="J63">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_66</t>
         </is>
       </c>
       <c r="J64">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_67</t>
         </is>
       </c>
       <c r="J65">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_68</t>
         </is>
       </c>
       <c r="J66">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_69</t>
         </is>
       </c>
       <c r="J67">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_7</t>
         </is>
       </c>
       <c r="J68">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_71</t>
         </is>
       </c>
       <c r="J69">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_72</t>
         </is>
       </c>
       <c r="J70">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_74</t>
         </is>
       </c>
       <c r="J71">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_75</t>
         </is>
       </c>
       <c r="J72">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_76</t>
         </is>
       </c>
       <c r="J73">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_77</t>
         </is>
       </c>
       <c r="J74">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_78</t>
         </is>
       </c>
       <c r="J75">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_80</t>
         </is>
       </c>
       <c r="J76">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_81</t>
         </is>
       </c>
       <c r="J77">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_82</t>
         </is>
       </c>
       <c r="J78">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_84</t>
         </is>
       </c>
       <c r="J79">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_89</t>
         </is>
       </c>
       <c r="J80">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_90</t>
         </is>
       </c>
       <c r="J81">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_91</t>
         </is>
       </c>
       <c r="J82">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_93</t>
         </is>
       </c>
       <c r="J83">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_94</t>
         </is>
       </c>
       <c r="J84">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_95</t>
         </is>
       </c>
       <c r="J85">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_96</t>
         </is>
       </c>
       <c r="J86">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>//1_//2</t>
+          <t>CBCL_97</t>
         </is>
       </c>
       <c r="J87">

</xml_diff>